<commit_message>
Initial commit - Tata Play Fiber project
</commit_message>
<xml_diff>
--- a/contacts.xlsx
+++ b/contacts.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
@@ -439,6 +439,33 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>2026-04-14 19:34:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Siddhantt</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>6226</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>patil123sidd@gmail.com</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>262</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-04-18 01:21:48</t>
         </is>
       </c>
     </row>

</xml_diff>